<commit_message>
Refresh S03-D1 evidence and record the second review round
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/evidence/s03d1/console/console_finance.xlsx
+++ b/evidence/s03d1/console/console_finance.xlsx
@@ -87,7 +87,7 @@
     <t>snapshot_id</t>
   </si>
   <si>
-    <t>3d1c342600421b956ad205c269c00408</t>
+    <t>98ba7ffc12463684e6ba95710026547a</t>
   </si>
   <si>
     <t>integration_id</t>
@@ -129,13 +129,13 @@
     <t>source_snapshot_ref</t>
   </si>
   <si>
-    <t>392ef306e69adef333e20efa41a5551f</t>
+    <t>e1317489f61c7fa78c0b910c94a53b1c</t>
   </si>
   <si>
     <t>expires_at</t>
   </si>
   <si>
-    <t>2026-10-27T01:50:43-06:00</t>
+    <t>2026-10-27T02:29:22-06:00</t>
   </si>
   <si>
     <t>precision</t>

</xml_diff>